<commit_message>
Added User Authentication, sign-up, sign-in logout
</commit_message>
<xml_diff>
--- a/01_Planning/Book1.xlsx
+++ b/01_Planning/Book1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="136">
   <si>
     <t>PROJECT PHASES</t>
   </si>
@@ -429,7 +429,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -446,12 +446,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -533,7 +527,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -559,13 +553,16 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
@@ -590,7 +587,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -897,10 +894,10 @@
   <dimension ref="A1:D72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="16" width="9.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="17" width="68.14785714285713" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="18" width="20.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="19" width="17.14785714285714" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="17" width="9.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="18" width="68.14785714285713" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="19" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="20" width="17.14785714285714" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -981,7 +978,7 @@
       <c r="C6" s="10">
         <v>3</v>
       </c>
-      <c r="D6" s="11"/>
+      <c r="D6" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="20.25">
       <c r="A7" s="7">
@@ -993,7 +990,7 @@
       <c r="C7" s="10">
         <v>3</v>
       </c>
-      <c r="D7" s="11"/>
+      <c r="D7" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="4" t="s">
@@ -1005,19 +1002,19 @@
       <c r="C8" s="6">
         <v>40</v>
       </c>
-      <c r="D8" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="12" t="s">
+      <c r="D8" s="12"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+      <c r="A9" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="15">
         <v>8</v>
       </c>
-      <c r="D9" s="11"/>
+      <c r="D9" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="7" t="s">
@@ -1029,7 +1026,9 @@
       <c r="C10" s="10">
         <v>1</v>
       </c>
-      <c r="D10" s="11"/>
+      <c r="D10" s="12" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="7" t="s">
@@ -1041,7 +1040,9 @@
       <c r="C11" s="10">
         <v>1</v>
       </c>
-      <c r="D11" s="11"/>
+      <c r="D11" s="12" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="7" t="s">
@@ -1053,7 +1054,9 @@
       <c r="C12" s="10">
         <v>2</v>
       </c>
-      <c r="D12" s="11"/>
+      <c r="D12" s="12" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="7" t="s">
@@ -1065,7 +1068,9 @@
       <c r="C13" s="10">
         <v>2</v>
       </c>
-      <c r="D13" s="11"/>
+      <c r="D13" s="12" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="20.25">
       <c r="A14" s="7" t="s">
@@ -1077,19 +1082,21 @@
       <c r="C14" s="10">
         <v>2</v>
       </c>
-      <c r="D14" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="12" t="s">
+      <c r="D14" s="12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
+      <c r="A15" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="15">
         <v>7</v>
       </c>
-      <c r="D15" s="11"/>
+      <c r="D15" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="7" t="s">
@@ -1101,7 +1108,7 @@
       <c r="C16" s="10">
         <v>2</v>
       </c>
-      <c r="D16" s="11"/>
+      <c r="D16" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="7" t="s">
@@ -1113,7 +1120,7 @@
       <c r="C17" s="10">
         <v>3</v>
       </c>
-      <c r="D17" s="11"/>
+      <c r="D17" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="7" t="s">
@@ -1125,7 +1132,7 @@
       <c r="C18" s="10">
         <v>1</v>
       </c>
-      <c r="D18" s="11"/>
+      <c r="D18" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="20.25">
       <c r="A19" s="7" t="s">
@@ -1137,19 +1144,19 @@
       <c r="C19" s="10">
         <v>1</v>
       </c>
-      <c r="D19" s="11"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="12" t="s">
+      <c r="D19" s="12"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
+      <c r="A20" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="B20" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="15">
         <v>6</v>
       </c>
-      <c r="D20" s="11"/>
+      <c r="D20" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="7" t="s">
@@ -1161,7 +1168,7 @@
       <c r="C21" s="10">
         <v>2</v>
       </c>
-      <c r="D21" s="11"/>
+      <c r="D21" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="7" t="s">
@@ -1173,7 +1180,7 @@
       <c r="C22" s="10">
         <v>2</v>
       </c>
-      <c r="D22" s="11"/>
+      <c r="D22" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="20.25">
       <c r="A23" s="7" t="s">
@@ -1185,19 +1192,19 @@
       <c r="C23" s="10">
         <v>2</v>
       </c>
-      <c r="D23" s="11"/>
+      <c r="D23" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="15">
         <v>9</v>
       </c>
-      <c r="D24" s="11"/>
+      <c r="D24" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
       <c r="A25" s="7" t="s">
@@ -1209,7 +1216,7 @@
       <c r="C25" s="10">
         <v>2</v>
       </c>
-      <c r="D25" s="11"/>
+      <c r="D25" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
       <c r="A26" s="7" t="s">
@@ -1221,7 +1228,7 @@
       <c r="C26" s="10">
         <v>3</v>
       </c>
-      <c r="D26" s="11"/>
+      <c r="D26" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
       <c r="A27" s="7" t="s">
@@ -1233,7 +1240,7 @@
       <c r="C27" s="10">
         <v>2</v>
       </c>
-      <c r="D27" s="11"/>
+      <c r="D27" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
       <c r="A28" s="7" t="s">
@@ -1245,19 +1252,19 @@
       <c r="C28" s="10">
         <v>2</v>
       </c>
-      <c r="D28" s="11"/>
+      <c r="D28" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="13" t="s">
+      <c r="B29" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C29" s="14">
+      <c r="C29" s="15">
         <v>5</v>
       </c>
-      <c r="D29" s="11"/>
+      <c r="D29" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
       <c r="A30" s="7" t="s">
@@ -1269,7 +1276,7 @@
       <c r="C30" s="10">
         <v>1</v>
       </c>
-      <c r="D30" s="11"/>
+      <c r="D30" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
       <c r="A31" s="7" t="s">
@@ -1281,7 +1288,7 @@
       <c r="C31" s="10">
         <v>2</v>
       </c>
-      <c r="D31" s="11"/>
+      <c r="D31" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
       <c r="A32" s="7" t="s">
@@ -1293,19 +1300,19 @@
       <c r="C32" s="10">
         <v>2</v>
       </c>
-      <c r="D32" s="11"/>
+      <c r="D32" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="B33" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C33" s="14">
+      <c r="C33" s="15">
         <v>9</v>
       </c>
-      <c r="D33" s="11"/>
+      <c r="D33" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="7" t="s">
@@ -1317,7 +1324,7 @@
       <c r="C34" s="10">
         <v>2</v>
       </c>
-      <c r="D34" s="11"/>
+      <c r="D34" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
       <c r="A35" s="7" t="s">
@@ -1329,7 +1336,7 @@
       <c r="C35" s="10">
         <v>2</v>
       </c>
-      <c r="D35" s="11"/>
+      <c r="D35" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
       <c r="A36" s="7" t="s">
@@ -1341,7 +1348,7 @@
       <c r="C36" s="10">
         <v>3</v>
       </c>
-      <c r="D36" s="11"/>
+      <c r="D36" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
       <c r="A37" s="7" t="s">
@@ -1353,7 +1360,7 @@
       <c r="C37" s="10">
         <v>2</v>
       </c>
-      <c r="D37" s="11"/>
+      <c r="D37" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
       <c r="A38" s="4" t="s">
@@ -1365,19 +1372,19 @@
       <c r="C38" s="6">
         <v>38</v>
       </c>
-      <c r="D38" s="11"/>
+      <c r="D38" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="12" t="s">
+      <c r="A39" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="B39" s="13" t="s">
+      <c r="B39" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="C39" s="14">
+      <c r="C39" s="15">
         <v>5</v>
       </c>
-      <c r="D39" s="11"/>
+      <c r="D39" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
       <c r="A40" s="7" t="s">
@@ -1389,7 +1396,7 @@
       <c r="C40" s="10">
         <v>1</v>
       </c>
-      <c r="D40" s="11"/>
+      <c r="D40" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
       <c r="A41" s="7" t="s">
@@ -1401,7 +1408,7 @@
       <c r="C41" s="10">
         <v>1</v>
       </c>
-      <c r="D41" s="11"/>
+      <c r="D41" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
       <c r="A42" s="7" t="s">
@@ -1413,19 +1420,19 @@
       <c r="C42" s="10">
         <v>3</v>
       </c>
-      <c r="D42" s="11"/>
+      <c r="D42" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
-      <c r="A43" s="12" t="s">
+      <c r="A43" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B43" s="13" t="s">
+      <c r="B43" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="C43" s="14">
+      <c r="C43" s="15">
         <v>14</v>
       </c>
-      <c r="D43" s="11"/>
+      <c r="D43" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
       <c r="A44" s="7" t="s">
@@ -1437,7 +1444,7 @@
       <c r="C44" s="10">
         <v>3</v>
       </c>
-      <c r="D44" s="11"/>
+      <c r="D44" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
       <c r="A45" s="7" t="s">
@@ -1449,7 +1456,7 @@
       <c r="C45" s="10">
         <v>3</v>
       </c>
-      <c r="D45" s="11"/>
+      <c r="D45" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
       <c r="A46" s="7" t="s">
@@ -1461,7 +1468,7 @@
       <c r="C46" s="10">
         <v>3</v>
       </c>
-      <c r="D46" s="11"/>
+      <c r="D46" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
       <c r="A47" s="7" t="s">
@@ -1473,7 +1480,7 @@
       <c r="C47" s="10">
         <v>3</v>
       </c>
-      <c r="D47" s="11"/>
+      <c r="D47" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
       <c r="A48" s="7" t="s">
@@ -1485,19 +1492,19 @@
       <c r="C48" s="10">
         <v>2</v>
       </c>
-      <c r="D48" s="11"/>
+      <c r="D48" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
-      <c r="A49" s="12" t="s">
+      <c r="A49" s="13" t="s">
         <v>93</v>
       </c>
-      <c r="B49" s="13" t="s">
+      <c r="B49" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="C49" s="14">
+      <c r="C49" s="15">
         <v>7</v>
       </c>
-      <c r="D49" s="11"/>
+      <c r="D49" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
       <c r="A50" s="7" t="s">
@@ -1509,7 +1516,7 @@
       <c r="C50" s="10">
         <v>2</v>
       </c>
-      <c r="D50" s="11"/>
+      <c r="D50" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
       <c r="A51" s="7" t="s">
@@ -1521,7 +1528,7 @@
       <c r="C51" s="10">
         <v>2</v>
       </c>
-      <c r="D51" s="11"/>
+      <c r="D51" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
       <c r="A52" s="7" t="s">
@@ -1533,7 +1540,7 @@
       <c r="C52" s="10">
         <v>2</v>
       </c>
-      <c r="D52" s="11"/>
+      <c r="D52" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
       <c r="A53" s="7" t="s">
@@ -1545,7 +1552,7 @@
       <c r="C53" s="10">
         <v>1</v>
       </c>
-      <c r="D53" s="11"/>
+      <c r="D53" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
       <c r="A54" s="4" t="s">
@@ -1557,19 +1564,19 @@
       <c r="C54" s="6">
         <v>20</v>
       </c>
-      <c r="D54" s="11"/>
+      <c r="D54" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
-      <c r="A55" s="12" t="s">
+      <c r="A55" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B55" s="13" t="s">
+      <c r="B55" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="C55" s="14">
+      <c r="C55" s="15">
         <v>8</v>
       </c>
-      <c r="D55" s="11"/>
+      <c r="D55" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
       <c r="A56" s="7" t="s">
@@ -1581,7 +1588,7 @@
       <c r="C56" s="10">
         <v>3</v>
       </c>
-      <c r="D56" s="11"/>
+      <c r="D56" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
       <c r="A57" s="7" t="s">
@@ -1593,7 +1600,7 @@
       <c r="C57" s="10">
         <v>2</v>
       </c>
-      <c r="D57" s="11"/>
+      <c r="D57" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
       <c r="A58" s="7" t="s">
@@ -1605,19 +1612,19 @@
       <c r="C58" s="10">
         <v>3</v>
       </c>
-      <c r="D58" s="11"/>
+      <c r="D58" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
-      <c r="A59" s="12" t="s">
+      <c r="A59" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="B59" s="13" t="s">
+      <c r="B59" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="C59" s="14">
+      <c r="C59" s="15">
         <v>6</v>
       </c>
-      <c r="D59" s="11"/>
+      <c r="D59" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
       <c r="A60" s="7" t="s">
@@ -1629,7 +1636,7 @@
       <c r="C60" s="10">
         <v>2</v>
       </c>
-      <c r="D60" s="11"/>
+      <c r="D60" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
       <c r="A61" s="7" t="s">
@@ -1641,7 +1648,7 @@
       <c r="C61" s="10">
         <v>2</v>
       </c>
-      <c r="D61" s="11"/>
+      <c r="D61" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
       <c r="A62" s="7" t="s">
@@ -1653,19 +1660,19 @@
       <c r="C62" s="10">
         <v>2</v>
       </c>
-      <c r="D62" s="11"/>
+      <c r="D62" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
-      <c r="A63" s="12" t="s">
+      <c r="A63" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="B63" s="13" t="s">
+      <c r="B63" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="C63" s="14">
+      <c r="C63" s="15">
         <v>6</v>
       </c>
-      <c r="D63" s="11"/>
+      <c r="D63" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
       <c r="A64" s="7" t="s">
@@ -1677,7 +1684,7 @@
       <c r="C64" s="10">
         <v>2</v>
       </c>
-      <c r="D64" s="11"/>
+      <c r="D64" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
       <c r="A65" s="7" t="s">
@@ -1689,7 +1696,7 @@
       <c r="C65" s="10">
         <v>2</v>
       </c>
-      <c r="D65" s="11"/>
+      <c r="D65" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
       <c r="A66" s="7" t="s">
@@ -1701,7 +1708,7 @@
       <c r="C66" s="10">
         <v>2</v>
       </c>
-      <c r="D66" s="11"/>
+      <c r="D66" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
       <c r="A67" s="4" t="s">
@@ -1713,7 +1720,7 @@
       <c r="C67" s="6">
         <v>14</v>
       </c>
-      <c r="D67" s="11"/>
+      <c r="D67" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
       <c r="A68" s="7">
@@ -1725,7 +1732,7 @@
       <c r="C68" s="10">
         <v>4</v>
       </c>
-      <c r="D68" s="11"/>
+      <c r="D68" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
       <c r="A69" s="7">
@@ -1737,7 +1744,7 @@
       <c r="C69" s="10">
         <v>3</v>
       </c>
-      <c r="D69" s="11"/>
+      <c r="D69" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
       <c r="A70" s="7">
@@ -1749,7 +1756,7 @@
       <c r="C70" s="10">
         <v>4</v>
       </c>
-      <c r="D70" s="11"/>
+      <c r="D70" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
       <c r="A71" s="7">
@@ -1761,7 +1768,7 @@
       <c r="C71" s="10">
         <v>3</v>
       </c>
-      <c r="D71" s="11"/>
+      <c r="D71" s="12"/>
     </row>
     <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
       <c r="A72" s="7">
@@ -1770,10 +1777,10 @@
       <c r="B72" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="C72" s="15">
+      <c r="C72" s="16">
         <v>0</v>
       </c>
-      <c r="D72" s="11"/>
+      <c r="D72" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>